<commit_message>
docs(revision): agenda con cierre anual, sobreprecio, fondos del caso y preguntas para las licenciadas
- Decisiones 15 a 18 (18 en total); decisión 3 solo HON-OTROS; decisión 4 con el mayor de
  QuickBooks de enero a julio.
- Sección 18: preguntas para las licenciadas (HON-FAM, tarjeta, sobreprecio).
- Excel NIIF: la lista queda con Operación, Inversión y Financiamiento.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/revision-josuarth/cuentas-de-resultado-niif.xlsx
+++ b/docs/revision-josuarth/cuentas-de-resultado-niif.xlsx
@@ -1338,7 +1338,7 @@
   </ignoredErrors>
   <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Opción no válida" error="Elige una opción de la lista." promptTitle="Tu clasificación" prompt="Elige una opción de la lista." sqref="E2:E46">
-      <formula1>"Operación,Inversión,Financiamiento,Impuestos,Operaciones discontinuadas"</formula1>
+      <formula1>"Operación,Inversión,Financiamiento"</formula1>
     </dataValidation>
   </dataValidations>
 </worksheet>
@@ -1408,7 +1408,7 @@
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>Opciones: Operación, Inversión, Financiamiento, Impuestos, Operaciones discontinuadas.</v>
+        <v>Opciones: Operación, Inversión, Financiamiento.</v>
       </c>
     </row>
   </sheetData>

</xml_diff>